<commit_message>
feat: add contact page, sitemap, and product URL redirects with tests
</commit_message>
<xml_diff>
--- a/indiarfidshop_SEO_Title_Audit.xlsx
+++ b/indiarfidshop_SEO_Title_Audit.xlsx
@@ -2016,7 +2016,7 @@
       </c>
       <c r="B7" s="3" t="n">
         <f aca="false">COUNTIF('All Pages'!K2:K50,"Needs fix")</f>
-        <v>48</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B12" s="3" t="n">
         <f aca="false">COUNTIFS(Issues!M2:M74,"&lt;&gt;Fixed",Issues!M2:M74,"&lt;&gt;Verified")</f>
-        <v>73</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2559,7 +2559,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="100"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2648,13 +2648,20 @@
         <f aca="false">IF(K2="","",LEN(K2))</f>
         <v>54</v>
       </c>
-      <c r="M2" s="13" t="s">
-        <v>63</v>
+      <c r="M2" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N2" s="13"/>
-      <c r="O2" s="13"/>
-    </row>
-    <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O2" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the homepage sets its own full title with the brand once (HOME_TITLE in src/lib/seo.ts).
+Checked live 9 Oct 2026: title is 'RFID Readers, Tags &amp; Antennas in India | Virtualsphere' (54 chars, brand once).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="54.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
         <v>64</v>
       </c>
@@ -2693,11 +2700,18 @@
         <f aca="false">IF(K3="","",LEN(K3))</f>
         <v>54</v>
       </c>
-      <c r="M3" s="13" t="s">
-        <v>63</v>
+      <c r="M3" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N3" s="13"/>
-      <c r="O3" s="13"/>
+      <c r="O3" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the homepage sets its own full title with the brand once (HOME_TITLE in src/lib/seo.ts).
+Checked live 9 Oct 2026: title is 'RFID Readers, Tags &amp; Antennas in India | Virtualsphere' (54 chars, brand once).</t>
+        </is>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
@@ -2738,11 +2752,18 @@
         <f aca="false">IF(K4="","",LEN(K4))</f>
         <v>32</v>
       </c>
-      <c r="M4" s="13" t="s">
-        <v>63</v>
+      <c r="M4" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N4" s="13"/>
-      <c r="O4" s="13"/>
+      <c r="O4" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): each category page gets its own title from CATEGORY_TITLES (src/app/(public)/products/page.tsx).
+Checked live 9 Oct 2026: title is 'Buy RFID Label Printers | Virtualsphere' (39 chars), unique among all pages. Wording differs from the suggestion ('Barcode Printers'); the category is now named RFID Printers.</t>
+        </is>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
@@ -2783,11 +2804,18 @@
         <f aca="false">IF(K5="","",LEN(K5))</f>
         <v>43</v>
       </c>
-      <c r="M5" s="13" t="s">
-        <v>63</v>
+      <c r="M5" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N5" s="13"/>
-      <c r="O5" s="13"/>
+      <c r="O5" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): each category page gets its own title from CATEGORY_TITLES (src/app/(public)/products/page.tsx).
+Checked live 9 Oct 2026: title is 'UHF Integrated RFID Readers | Virtualsphere' (43 chars), unique among all pages.</t>
+        </is>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
@@ -2828,11 +2856,18 @@
         <f aca="false">IF(K6="","",LEN(K6))</f>
         <v>45</v>
       </c>
-      <c r="M6" s="13" t="s">
-        <v>63</v>
+      <c r="M6" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N6" s="13"/>
-      <c r="O6" s="13"/>
+      <c r="O6" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): each category page gets its own title from CATEGORY_TITLES (src/app/(public)/products/page.tsx).
+Checked live 9 Oct 2026: title is '4-Port UHF RFID Fixed Readers | Virtualsphere' (45 chars), unique among all pages.</t>
+        </is>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
@@ -2873,11 +2908,18 @@
         <f aca="false">IF(K7="","",LEN(K7))</f>
         <v>46</v>
       </c>
-      <c r="M7" s="13" t="s">
-        <v>63</v>
+      <c r="M7" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N7" s="13"/>
-      <c r="O7" s="13"/>
+      <c r="O7" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): each category page gets its own title from CATEGORY_TITLES (src/app/(public)/products/page.tsx).
+Checked live 9 Oct 2026: title is 'RFID Tags – UHF, HF &amp; On-Metal | Virtualsphere' (46 chars), unique among all pages. Checked at the renamed URL /products?category=rfid-tags (see T038).</t>
+        </is>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
@@ -2918,11 +2960,18 @@
         <f aca="false">IF(K8="","",LEN(K8))</f>
         <v>31</v>
       </c>
-      <c r="M8" s="13" t="s">
-        <v>63</v>
+      <c r="M8" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N8" s="13"/>
-      <c r="O8" s="13"/>
+      <c r="O8" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): each category page gets its own title from CATEGORY_TITLES (src/app/(public)/products/page.tsx).
+Checked live 9 Oct 2026: title is 'UHF RFID Labels | Virtualsphere' (31 chars), unique among all pages.</t>
+        </is>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
@@ -2963,11 +3012,18 @@
         <f aca="false">IF(K9="","",LEN(K9))</f>
         <v>33</v>
       </c>
-      <c r="M9" s="13" t="s">
-        <v>63</v>
+      <c r="M9" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N9" s="13"/>
-      <c r="O9" s="13"/>
+      <c r="O9" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): each category page gets its own title from CATEGORY_TITLES (src/app/(public)/products/page.tsx).
+Checked live 9 Oct 2026: title is 'RFID Laundry Tags | Virtualsphere' (33 chars), unique among all pages. Checked at the renamed URL /products?category=rfid-laundry-tags (see T039).</t>
+        </is>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
@@ -3008,11 +3064,18 @@
         <f aca="false">IF(K10="","",LEN(K10))</f>
         <v>43</v>
       </c>
-      <c r="M10" s="13" t="s">
-        <v>63</v>
+      <c r="M10" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N10" s="13"/>
-      <c r="O10" s="13"/>
+      <c r="O10" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): each category page gets its own title from CATEGORY_TITLES (src/app/(public)/products/page.tsx).
+Checked live 9 Oct 2026: title is 'UHF RFID Inlays - Dry &amp; Wet | Virtualsphere' (43 chars), unique among all pages. Same text as suggested but with a hyphen instead of the en dash.</t>
+        </is>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
@@ -3053,11 +3116,18 @@
         <f aca="false">IF(K11="","",LEN(K11))</f>
         <v>38</v>
       </c>
-      <c r="M11" s="13" t="s">
-        <v>63</v>
+      <c r="M11" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N11" s="13"/>
-      <c r="O11" s="13"/>
+      <c r="O11" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): each category page gets its own title from CATEGORY_TITLES (src/app/(public)/products/page.tsx).
+Checked live 9 Oct 2026: title is 'UHF RFID ABS Hard Tags | Virtualsphere' (38 chars), unique among all pages.</t>
+        </is>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
@@ -3098,11 +3168,18 @@
         <f aca="false">IF(K12="","",LEN(K12))</f>
         <v>33</v>
       </c>
-      <c r="M12" s="13" t="s">
-        <v>63</v>
+      <c r="M12" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N12" s="13"/>
-      <c r="O12" s="13"/>
+      <c r="O12" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): each category page gets its own title from CATEGORY_TITLES (src/app/(public)/products/page.tsx).
+Checked live 9 Oct 2026: title is 'UHF RFID Antennas | Virtualsphere' (33 chars), unique among all pages.</t>
+        </is>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
@@ -3143,11 +3220,18 @@
         <f aca="false">IF(K13="","",LEN(K13))</f>
         <v>41</v>
       </c>
-      <c r="M13" s="13" t="s">
-        <v>63</v>
+      <c r="M13" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N13" s="13"/>
-      <c r="O13" s="13"/>
+      <c r="O13" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): each category page gets its own title from CATEGORY_TITLES (src/app/(public)/products/page.tsx).
+Checked live 9 Oct 2026: title is 'UHF RFID Handheld Readers | Virtualsphere' (41 chars), unique among all pages.</t>
+        </is>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
@@ -3188,11 +3272,18 @@
         <f aca="false">IF(K14="","",LEN(K14))</f>
         <v>50</v>
       </c>
-      <c r="M14" s="13" t="s">
-        <v>63</v>
+      <c r="M14" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N14" s="13"/>
-      <c r="O14" s="13"/>
+      <c r="O14" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): each category page gets its own title from CATEGORY_TITLES (src/app/(public)/products/page.tsx).
+Checked live 9 Oct 2026: title is 'UHF RFID Desktop Readers &amp; Writers | Virtualsphere' (50 chars), unique among all pages.</t>
+        </is>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
@@ -3233,11 +3324,18 @@
         <f aca="false">IF(K15="","",LEN(K15))</f>
         <v>41</v>
       </c>
-      <c r="M15" s="13" t="s">
-        <v>63</v>
+      <c r="M15" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N15" s="13"/>
-      <c r="O15" s="13"/>
+      <c r="O15" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): each category page gets its own title from CATEGORY_TITLES (src/app/(public)/products/page.tsx).
+Checked live 9 Oct 2026: title is 'HF 13.56 MHz RFID Readers | Virtualsphere' (41 chars), unique among all pages.</t>
+        </is>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
@@ -3278,11 +3376,18 @@
         <f aca="false">IF(K16="","",LEN(K16))</f>
         <v>49</v>
       </c>
-      <c r="M16" s="13" t="s">
-        <v>63</v>
+      <c r="M16" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N16" s="13"/>
-      <c r="O16" s="13"/>
+      <c r="O16" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): each category page gets its own title from CATEGORY_TITLES (src/app/(public)/products/page.tsx).
+Checked live 9 Oct 2026: title is 'LF &amp; HF RFID USB Pendrive Readers | Virtualsphere' (49 chars), unique among all pages.</t>
+        </is>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
@@ -3323,11 +3428,18 @@
         <f aca="false">IF(K17="","",LEN(K17))</f>
         <v>45</v>
       </c>
-      <c r="M17" s="13" t="s">
-        <v>63</v>
+      <c r="M17" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N17" s="13"/>
-      <c r="O17" s="13"/>
+      <c r="O17" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the product title is set in PRODUCT_TITLES (src/app/(public)/products/[slug]/page.tsx); the layout adds the brand once and a stored '| Virtualsphere' is stripped (stripBrand, src/lib/seo.ts).
+Checked live 9 Oct 2026: title is 'Desktop Barcode Label Printer | Virtualsphere' (45 chars, brand once).</t>
+        </is>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
@@ -3368,11 +3480,18 @@
         <f aca="false">IF(K18="","",LEN(K18))</f>
         <v>58</v>
       </c>
-      <c r="M18" s="13" t="s">
-        <v>63</v>
+      <c r="M18" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N18" s="13"/>
-      <c r="O18" s="13"/>
+      <c r="O18" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the product title is set in PRODUCT_TITLES (src/app/(public)/products/[slug]/page.tsx); the layout adds the brand once and a stored '| Virtualsphere' is stripped (stripBrand, src/lib/seo.ts).
+Checked live 9 Oct 2026: title is 'HRD 13 HF 13.56MHz USB Desktop RFID Reader | Virtualsphere' (58 chars, brand once).</t>
+        </is>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
@@ -3413,11 +3532,18 @@
         <f aca="false">IF(K19="","",LEN(K19))</f>
         <v>57</v>
       </c>
-      <c r="M19" s="13" t="s">
-        <v>63</v>
+      <c r="M19" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N19" s="13"/>
-      <c r="O19" s="13"/>
+      <c r="O19" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the product title is set in PRODUCT_TITLES (src/app/(public)/products/[slug]/page.tsx); the layout adds the brand once and a stored '| Virtualsphere' is stripped (stripBrand, src/lib/seo.ts).
+Checked live 9 Oct 2026: title is 'LRP 70 125KHz LF RFID USB Pendrive Reader | Virtualsphere' (57 chars, brand once).</t>
+        </is>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
@@ -3458,11 +3584,18 @@
         <f aca="false">IF(K20="","",LEN(K20))</f>
         <v>56</v>
       </c>
-      <c r="M20" s="13" t="s">
-        <v>63</v>
+      <c r="M20" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N20" s="13"/>
-      <c r="O20" s="13"/>
+      <c r="O20" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the product title is set in PRODUCT_TITLES (src/app/(public)/products/[slug]/page.tsx); the layout adds the brand once and a stored '| Virtualsphere' is stripped (stripBrand, src/lib/seo.ts).
+Checked live 9 Oct 2026: title is 'UA9 9dBi Circular UHF RFID Antenna, IP67 | Virtualsphere' (56 chars, brand once).</t>
+        </is>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
@@ -3503,11 +3636,18 @@
         <f aca="false">IF(K21="","",LEN(K21))</f>
         <v>56</v>
       </c>
-      <c r="M21" s="13" t="s">
-        <v>63</v>
+      <c r="M21" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N21" s="13"/>
-      <c r="O21" s="13"/>
+      <c r="O21" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the product title is set in PRODUCT_TITLES (src/app/(public)/products/[slug]/page.tsx); the layout adds the brand once and a stored '| Virtualsphere' is stripped (stripBrand, src/lib/seo.ts).
+Checked live 9 Oct 2026: title is 'UCA3 3dBi Ceramic UHF RFID Patch Antenna | Virtualsphere' (56 chars, brand once).</t>
+        </is>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
@@ -3548,11 +3688,18 @@
         <f aca="false">IF(K22="","",LEN(K22))</f>
         <v>57</v>
       </c>
-      <c r="M22" s="13" t="s">
-        <v>63</v>
+      <c r="M22" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N22" s="13"/>
-      <c r="O22" s="13"/>
+      <c r="O22" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the product title is set in PRODUCT_TITLES (src/app/(public)/products/[slug]/page.tsx); the layout adds the brand once and a stored '| Virtualsphere' is stripped (stripBrand, src/lib/seo.ts).
+Checked live 9 Oct 2026: title is 'UDR-W101 UHF RFID Desktop Reader &amp; Writer | Virtualsphere' (57 chars, brand once).</t>
+        </is>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
@@ -3593,11 +3740,18 @@
         <f aca="false">IF(K23="","",LEN(K23))</f>
         <v>59</v>
       </c>
-      <c r="M23" s="13" t="s">
-        <v>63</v>
+      <c r="M23" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N23" s="13"/>
-      <c r="O23" s="13"/>
+      <c r="O23" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the product title is set in PRODUCT_TITLES (src/app/(public)/products/[slug]/page.tsx); the layout adds the brand once and a stored '| Virtualsphere' is stripped (stripBrand, src/lib/seo.ts).
+Checked live 9 Oct 2026: title is 'UDT9R RFID Jewellery Tray Reader, Bluetooth | Virtualsphere' (59 chars, brand once).</t>
+        </is>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
@@ -3638,11 +3792,18 @@
         <f aca="false">IF(K24="","",LEN(K24))</f>
         <v>58</v>
       </c>
-      <c r="M24" s="13" t="s">
-        <v>63</v>
+      <c r="M24" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N24" s="13"/>
-      <c r="O24" s="13"/>
+      <c r="O24" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the product title is set in PRODUCT_TITLES (src/app/(public)/products/[slug]/page.tsx); the layout adds the brand once and a stored '| Virtualsphere' is stripped (stripBrand, src/lib/seo.ts).
+Checked live 9 Oct 2026: title is 'UHR2 Android UHF RFID Handheld Reader, 20m | Virtualsphere' (58 chars, brand once).</t>
+        </is>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
@@ -3683,11 +3844,18 @@
         <f aca="false">IF(K25="","",LEN(K25))</f>
         <v>54</v>
       </c>
-      <c r="M25" s="13" t="s">
-        <v>63</v>
+      <c r="M25" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N25" s="13"/>
-      <c r="O25" s="13"/>
+      <c r="O25" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the product title is set in PRODUCT_TITLES (src/app/(public)/products/[slug]/page.tsx); the layout adds the brand once and a stored '| Virtualsphere' is stripped (stripBrand, src/lib/seo.ts).
+Checked live 9 Oct 2026: title is 'VST-9662 UHF RFID Inlay, Alien Higgs-3 | Virtualsphere' (54 chars, brand once).</t>
+        </is>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
@@ -3728,11 +3896,18 @@
         <f aca="false">IF(K26="","",LEN(K26))</f>
         <v>55</v>
       </c>
-      <c r="M26" s="13" t="s">
-        <v>63</v>
+      <c r="M26" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N26" s="13"/>
-      <c r="O26" s="13"/>
+      <c r="O26" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the product title is set in PRODUCT_TITLES (src/app/(public)/products/[slug]/page.tsx); the layout adds the brand once and a stored '| Virtualsphere' is stripped (stripBrand, src/lib/seo.ts).
+Checked live 9 Oct 2026: title is 'PBR3 Bluetooth UHF RFID Portable Reader | Virtualsphere' (55 chars, brand once).</t>
+        </is>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
@@ -3773,11 +3948,18 @@
         <f aca="false">IF(K27="","",LEN(K27))</f>
         <v>52</v>
       </c>
-      <c r="M27" s="13" t="s">
-        <v>63</v>
+      <c r="M27" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N27" s="13"/>
-      <c r="O27" s="13"/>
+      <c r="O27" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the product title is set in PRODUCT_TITLES (src/app/(public)/products/[slug]/page.tsx); the layout adds the brand once and a stored '| Virtualsphere' is stripped (stripBrand, src/lib/seo.ts).
+Checked live 9 Oct 2026: title is 'UA12 12dBi Circular UHF RFID Antenna | Virtualsphere' (52 chars, brand once).</t>
+        </is>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
@@ -3818,13 +4000,20 @@
         <f aca="false">IF(K28="","",LEN(K28))</f>
         <v>55</v>
       </c>
-      <c r="M28" s="13" t="s">
-        <v>63</v>
+      <c r="M28" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N28" s="13"/>
-      <c r="O28" s="13"/>
-    </row>
-    <row r="29" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O28" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the product title is set in PRODUCT_TITLES (src/app/(public)/products/[slug]/page.tsx); the layout adds the brand once and a stored '| Virtualsphere' is stripped (stripBrand, src/lib/seo.ts).
+Checked live 9 Oct 2026: title is 'UHR 5 UHF RFID Handheld Reader with NFC | Virtualsphere' (55 chars, brand once).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="67.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
         <v>196</v>
       </c>
@@ -3863,13 +4052,20 @@
         <f aca="false">IF(K29="","",LEN(K29))</f>
         <v>58</v>
       </c>
-      <c r="M29" s="13" t="s">
-        <v>63</v>
+      <c r="M29" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N29" s="13"/>
-      <c r="O29" s="13"/>
-    </row>
-    <row r="30" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O29" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the product title is set in PRODUCT_TITLES (src/app/(public)/products/[slug]/page.tsx); the layout adds the brand once and a stored '| Virtualsphere' is stripped (stripBrand, src/lib/seo.ts).
+Checked live 9 Oct 2026: title is 'HRD 13 HF 13.56MHz USB Desktop RFID Reader | Virtualsphere' (58 chars, brand once).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="67.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
         <v>199</v>
       </c>
@@ -3908,13 +4104,20 @@
         <f aca="false">IF(K30="","",LEN(K30))</f>
         <v>56</v>
       </c>
-      <c r="M30" s="13" t="s">
-        <v>63</v>
+      <c r="M30" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N30" s="13"/>
-      <c r="O30" s="13"/>
-    </row>
-    <row r="31" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O30" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the product title is set in PRODUCT_TITLES (src/app/(public)/products/[slug]/page.tsx); the layout adds the brand once and a stored '| Virtualsphere' is stripped (stripBrand, src/lib/seo.ts).
+Checked live 9 Oct 2026: title is 'UA9 9dBi Circular UHF RFID Antenna, IP67 | Virtualsphere' (56 chars, brand once).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="67.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
         <v>200</v>
       </c>
@@ -3953,13 +4156,20 @@
         <f aca="false">IF(K31="","",LEN(K31))</f>
         <v>56</v>
       </c>
-      <c r="M31" s="13" t="s">
-        <v>63</v>
+      <c r="M31" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N31" s="13"/>
-      <c r="O31" s="13"/>
-    </row>
-    <row r="32" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O31" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the product title is set in PRODUCT_TITLES (src/app/(public)/products/[slug]/page.tsx); the layout adds the brand once and a stored '| Virtualsphere' is stripped (stripBrand, src/lib/seo.ts).
+Checked live 9 Oct 2026: title is 'UCA3 3dBi Ceramic UHF RFID Patch Antenna | Virtualsphere' (56 chars, brand once).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="67.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
         <v>201</v>
       </c>
@@ -3998,13 +4208,20 @@
         <f aca="false">IF(K32="","",LEN(K32))</f>
         <v>57</v>
       </c>
-      <c r="M32" s="13" t="s">
-        <v>63</v>
+      <c r="M32" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N32" s="13"/>
-      <c r="O32" s="13"/>
-    </row>
-    <row r="33" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O32" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the product title is set in PRODUCT_TITLES (src/app/(public)/products/[slug]/page.tsx); the layout adds the brand once and a stored '| Virtualsphere' is stripped (stripBrand, src/lib/seo.ts).
+Checked live 9 Oct 2026: title is 'LRP 70 125KHz LF RFID USB Pendrive Reader | Virtualsphere' (57 chars, brand once).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="67.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
         <v>202</v>
       </c>
@@ -4043,13 +4260,20 @@
         <f aca="false">IF(K33="","",LEN(K33))</f>
         <v>55</v>
       </c>
-      <c r="M33" s="13" t="s">
-        <v>63</v>
+      <c r="M33" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N33" s="13"/>
-      <c r="O33" s="13"/>
-    </row>
-    <row r="34" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O33" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the product title is set in PRODUCT_TITLES (src/app/(public)/products/[slug]/page.tsx); the layout adds the brand once and a stored '| Virtualsphere' is stripped (stripBrand, src/lib/seo.ts).
+Checked live 9 Oct 2026: title is 'UHR 5 UHF RFID Handheld Reader with NFC | Virtualsphere' (55 chars, brand once).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="67.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
         <v>205</v>
       </c>
@@ -4088,11 +4312,18 @@
         <f aca="false">IF(K34="","",LEN(K34))</f>
         <v>56</v>
       </c>
-      <c r="M34" s="13" t="s">
-        <v>63</v>
+      <c r="M34" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N34" s="13"/>
-      <c r="O34" s="13"/>
+      <c r="O34" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit de884b4, 7 Oct): the product title is set in PRODUCT_TITLES (src/app/(public)/products/[slug]/page.tsx); the layout adds the brand once and a stored '| Virtualsphere' is stripped (stripBrand, src/lib/seo.ts).
+Checked live 9 Oct 2026: title is 'UDR 102 UHF RFID Desktop Reader &amp; Writer | Virtualsphere' (56 chars, brand once).</t>
+        </is>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
@@ -4123,13 +4354,20 @@
       <c r="J35" s="10"/>
       <c r="K35" s="10"/>
       <c r="L35" s="12"/>
-      <c r="M35" s="13" t="s">
-        <v>63</v>
+      <c r="M35" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N35" s="13"/>
-      <c r="O35" s="13"/>
-    </row>
-    <row r="36" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O35" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): every page sets its own canonical URL (pageMetadata in src/lib/seo.ts).
+Checked live 9 Oct 2026: 49 of 49 sitemap URLs carry an absolute https canonical link.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="54.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
         <v>217</v>
       </c>
@@ -4168,11 +4406,18 @@
         <f aca="false">IF(K36="","",LEN(K36))</f>
         <v>56</v>
       </c>
-      <c r="M36" s="13" t="s">
-        <v>63</v>
+      <c r="M36" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N36" s="13"/>
-      <c r="O36" s="13"/>
+      <c r="O36" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the /products title is set in src/app/(public)/products/page.tsx.
+Checked live 9 Oct 2026: title is 'Buy RFID Readers, Tags &amp; Antennas Online | Virtualsphere' (56 chars, brand once).</t>
+        </is>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
@@ -4213,11 +4458,18 @@
         <f aca="false">IF(K37="","",LEN(K37))</f>
         <v>30</v>
       </c>
-      <c r="M37" s="13" t="s">
-        <v>63</v>
+      <c r="M37" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N37" s="13"/>
-      <c r="O37" s="13"/>
+      <c r="O37" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the page title is set without the brand and the layout adds it once.
+Checked live 9 Oct 2026: title is 'Privacy Policy | Virtualsphere' (30 chars, brand once).</t>
+        </is>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
@@ -4258,13 +4510,20 @@
         <f aca="false">IF(K38="","",LEN(K38))</f>
         <v>34</v>
       </c>
-      <c r="M38" s="13" t="s">
-        <v>63</v>
+      <c r="M38" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N38" s="13"/>
-      <c r="O38" s="13"/>
-    </row>
-    <row r="39" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O38" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the page title is set without the brand and the layout adds it once.
+Checked live 9 Oct 2026: title is 'Terms &amp; Conditions | Virtualsphere' (34 chars, brand once).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="93.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
         <v>233</v>
       </c>
@@ -4297,13 +4556,25 @@
       </c>
       <c r="K39" s="10"/>
       <c r="L39" s="12"/>
-      <c r="M39" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N39" s="13"/>
-      <c r="O39" s="13"/>
-    </row>
-    <row r="40" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M39" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N39" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O39" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: category slug raid-tags changed to rfid-tags in the live catalog (admin API). Added a 301 redirect from the old URL to the new one (next.config.ts, commit c912301, deployed). No page hard-codes the old slug; links and the sitemap follow the catalog.
+Verified live: raid-tags URL answers 301 -&gt; /products?category=rfid-tags; the new URL loads with heading 'RFID Tags' and canonical https://indiarfidshop.com/products?category=rfid-tags; sitemap lists the new slug only.
+Still to do by site owner: resubmit the sitemap in Search Console.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="106.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="10" t="s">
         <v>237</v>
       </c>
@@ -4336,13 +4607,25 @@
       </c>
       <c r="K40" s="10"/>
       <c r="L40" s="12"/>
-      <c r="M40" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N40" s="13"/>
-      <c r="O40" s="13"/>
-    </row>
-    <row r="41" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M40" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N40" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O40" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: category renamed from 'RFID Laundary Tags' to 'RFID Laundry Tags' and its slug rfid-laundary-tags changed to rfid-laundry-tags in the live catalog (admin API); it stays under RFID Tags. Added a 301 redirect from the old URL to the new one (next.config.ts, commit c912301, deployed). No page hard-codes the old slug; links and the sitemap follow the catalog.
+Verified live: rfid-laundary-tags URL answers 301 -&gt; /products?category=rfid-laundry-tags; the new URL loads with heading 'RFID Laundry Tags' and canonical https://indiarfidshop.com/products?category=rfid-laundry-tags; sitemap lists the new slug only.
+Still to do by site owner: resubmit the sitemap in Search Console.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="67.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="10" t="s">
         <v>240</v>
       </c>
@@ -4375,13 +4658,24 @@
       </c>
       <c r="K41" s="10"/>
       <c r="L41" s="12"/>
-      <c r="M41" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N41" s="13"/>
-      <c r="O41" s="13"/>
-    </row>
-    <row r="42" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M41" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N41" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O41" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: product name (the H1) changed in the live catalog from 'UDR-W101 RFID Desktop Reader &amp; Writer | Virtualsphere' to 'UDR-W101 RFID Desktop Reader &amp; Writer'. Also added a guard (cleanProductName, commit c912301, deployed) so a brand suffix or pipe typed into a product name is cleaned before it reaches the heading, product cards and cart.
+Verified live: the page has exactly one H1: 'UDR-W101 RFID Desktop Reader &amp; Writer'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="67.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="10" t="s">
         <v>245</v>
       </c>
@@ -4414,13 +4708,24 @@
       </c>
       <c r="K42" s="10"/>
       <c r="L42" s="12"/>
-      <c r="M42" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N42" s="13"/>
-      <c r="O42" s="13"/>
-    </row>
-    <row r="43" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M42" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N42" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O42" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: product name (the H1) changed in the live catalog from 'UDT9R RFID Jewellery Tray Reader | Virtualsphere' to 'UDT9R RFID Jewellery Tray Reader'. Also added a guard (cleanProductName, commit c912301, deployed) so a brand suffix or pipe typed into a product name is cleaned before it reaches the heading, product cards and cart.
+Verified live: the page has exactly one H1: 'UDT9R RFID Jewellery Tray Reader'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="67.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="10" t="s">
         <v>247</v>
       </c>
@@ -4453,13 +4758,24 @@
       </c>
       <c r="K43" s="10"/>
       <c r="L43" s="12"/>
-      <c r="M43" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N43" s="13"/>
-      <c r="O43" s="13"/>
-    </row>
-    <row r="44" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M43" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N43" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O43" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: product name (the H1) changed in the live catalog from 'UHR2 UHF RFID Handheld Reader | Virtualsphere' to 'UHR2 UHF RFID Handheld Reader'. Also added a guard (cleanProductName, commit c912301, deployed) so a brand suffix or pipe typed into a product name is cleaned before it reaches the heading, product cards and cart.
+Verified live: the page has exactly one H1: 'UHR2 UHF RFID Handheld Reader'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="67.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="10" t="s">
         <v>249</v>
       </c>
@@ -4492,13 +4808,24 @@
       </c>
       <c r="K44" s="10"/>
       <c r="L44" s="12"/>
-      <c r="M44" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N44" s="13"/>
-      <c r="O44" s="13"/>
-    </row>
-    <row r="45" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M44" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N44" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O44" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: product name (the H1) changed in the live catalog from 'VSL-F2 UHF RFID 4 Port Reader | Impinj E710' to 'VSL-F2 UHF RFID 4 Port Reader – Impinj E710'. Also added a guard (cleanProductName, commit c912301, deployed) so a brand suffix or pipe typed into a product name is cleaned before it reaches the heading, product cards and cart.
+Verified live: the page has exactly one H1: 'VSL-F2 UHF RFID 4 Port Reader – Impinj E710'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="67.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="10" t="s">
         <v>253</v>
       </c>
@@ -4531,13 +4858,24 @@
       </c>
       <c r="K45" s="10"/>
       <c r="L45" s="12"/>
-      <c r="M45" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N45" s="13"/>
-      <c r="O45" s="13"/>
-    </row>
-    <row r="46" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M45" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N45" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O45" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: meta description replaced in the live catalog (was 'RFID Handheld Reader | UHR 72') with the suggested text, 144 characters.
+Verified live: &lt;meta name="description"&gt; in the page source reads 'Buy the UHR 72 UHF RFID handheld reader – EPC Gen2 / ISO 18000-6C with Gen2v2 authentication. Ideal for inventory, warehouse and asset tracking.'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="67.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="10" t="s">
         <v>259</v>
       </c>
@@ -4570,13 +4908,24 @@
       </c>
       <c r="K46" s="10"/>
       <c r="L46" s="12"/>
-      <c r="M46" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N46" s="13"/>
-      <c r="O46" s="13"/>
-    </row>
-    <row r="47" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M46" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N46" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O46" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: meta description replaced in the live catalog (was 'Virtualsphere UDM9R is a high-performance single-channel fixed RFID reader.') with the suggested text, 139 characters.
+Verified live: &lt;meta name="description"&gt; in the page source reads 'UDM9R long range integrated UHF RFID reader with Impinj E310, 9dBi antenna, up to 15 m range, IP68, RS232, RJ45, Wiegand &amp; GPIO interfaces.'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="67.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="10" t="s">
         <v>264</v>
       </c>
@@ -4609,13 +4958,24 @@
       </c>
       <c r="K47" s="10"/>
       <c r="L47" s="12"/>
-      <c r="M47" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N47" s="13"/>
-      <c r="O47" s="13"/>
-    </row>
-    <row r="48" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M47" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N47" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O47" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: meta description replaced in the live catalog (was 'Virtualsphere UDM12R is a high-performance single-channel fixed RFID reader.') with the suggested text, 144 characters.
+Verified live: &lt;meta name="description"&gt; in the page source reads 'UDM12R Impinj-based integrated UHF RFID reader, EPC Gen2 V2, read range up to 20 m, RS232, RJ45 &amp; GPIO – for access control, logistics &amp; assets.'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="93.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="10" t="s">
         <v>269</v>
       </c>
@@ -4648,13 +5008,24 @@
       </c>
       <c r="K48" s="10"/>
       <c r="L48" s="12"/>
-      <c r="M48" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N48" s="13"/>
-      <c r="O48" s="13"/>
-    </row>
-    <row r="49" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M48" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N48" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O48" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: meta description replaced in the live catalog (was '10-15mtrs Reader Long range desktop operating reader') with the suggested text, 155 characters. The wording says 'up to 7 m (23 ft)' instead of the suggested '10–15 m' because the product page itself says 23 feet; chosen by the site owner.
+Verified live: &lt;meta name="description"&gt; in the page source reads 'UDR 107 long range UHF RFID desktop reader with up to 7 m (23 ft) read range for gates, counters and inventory points. Easy integration with your software.'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="67.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="10" t="s">
         <v>274</v>
       </c>
@@ -4687,13 +5058,24 @@
       </c>
       <c r="K49" s="10"/>
       <c r="L49" s="12"/>
-      <c r="M49" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N49" s="13"/>
-      <c r="O49" s="13"/>
-    </row>
-    <row r="50" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M49" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N49" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O49" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: meta description replaced in the live catalog (was 'RFID Pendrive Reader | 13.56Mhz Reader | Portable Reader') with the suggested text, 138 characters.
+Verified live: &lt;meta name="description"&gt; in the page source reads 'HRP 70 driver-free 13.56MHz HF RFID USB pendrive reader, up to 80 mm range, IP65. Plug-and-play for access cards, attendance and NFC tags.'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="67.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="10" t="s">
         <v>279</v>
       </c>
@@ -4726,13 +5108,24 @@
       </c>
       <c r="K50" s="10"/>
       <c r="L50" s="12"/>
-      <c r="M50" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N50" s="13"/>
-      <c r="O50" s="13"/>
-    </row>
-    <row r="51" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M50" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N50" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O50" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: meta description replaced in the live catalog (was a 294-character copy of the product description, with line breaks) with the suggested text, 138 characters.
+Verified live: &lt;meta name="description"&gt; in the page source reads 'UDR 102 UHF RFID desktop reader &amp; writer with 3–5 m range for POS, registration and inventory. Works with Windows, iOS, Android and Linux.'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="67.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="10" t="s">
         <v>282</v>
       </c>
@@ -4761,13 +5154,20 @@
       <c r="J51" s="10"/>
       <c r="K51" s="10"/>
       <c r="L51" s="12"/>
-      <c r="M51" s="13" t="s">
-        <v>63</v>
+      <c r="M51" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N51" s="13"/>
-      <c r="O51" s="13"/>
-    </row>
-    <row r="52" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O51" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already correct on 9 Oct 2026, no change needed: every page sets its own og:title, og:url and twitter tags (pageMetadata in src/lib/seo.ts, added in commit 09f194b, 7 Oct).
+Checked live 9 Oct 2026: /, /products, a category page, /categories, /about, /contact, /privacy and /terms each carry a page-specific og:title (for example 'RFID Readers, Tags &amp; Antennas in India | Virtualsphere') and none the old generic one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="67.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="10" t="s">
         <v>286</v>
       </c>
@@ -4796,13 +5196,20 @@
       <c r="J52" s="10"/>
       <c r="K52" s="10"/>
       <c r="L52" s="12"/>
-      <c r="M52" s="13" t="s">
-        <v>63</v>
+      <c r="M52" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N52" s="13"/>
-      <c r="O52" s="13"/>
-    </row>
-    <row r="53" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O52" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already correct on 9 Oct 2026, no change needed: product pages set twitter:title/description and the og tags from the product's own title, description and image (pageMetadata, commit 09f194b, 7 Oct).
+Checked live 9 Oct 2026: the UDM9R page has twitter:title 'UDM9R Long Range Integrated UHF RFID Reader | Virtualsphere'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="54.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="10" t="s">
         <v>290</v>
       </c>
@@ -4831,13 +5238,20 @@
       <c r="J53" s="10"/>
       <c r="K53" s="10"/>
       <c r="L53" s="12"/>
-      <c r="M53" s="13" t="s">
-        <v>63</v>
+      <c r="M53" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N53" s="13"/>
-      <c r="O53" s="13"/>
-    </row>
-    <row r="54" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O53" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Could not reproduce on 9 Oct 2026, no change needed: the page is a server component with the full text written in it and no client-side fetch (it was already built this way before 7 Oct), so the server HTML contains the text (about 828 words).
+Checked live 9 Oct 2026: the opening sentence is present in the raw HTML.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="54.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="10" t="s">
         <v>293</v>
       </c>
@@ -4866,13 +5280,20 @@
       <c r="J54" s="10"/>
       <c r="K54" s="10"/>
       <c r="L54" s="12"/>
-      <c r="M54" s="13" t="s">
-        <v>63</v>
+      <c r="M54" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N54" s="13"/>
-      <c r="O54" s="13"/>
-    </row>
-    <row r="55" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O54" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Could not reproduce on 9 Oct 2026, no change needed: the page is a server component with the full text written in it and no client-side fetch (it was already built this way before 7 Oct), so the server HTML contains the text (about 549 words).
+Checked live 9 Oct 2026: the opening sentence is present in the raw HTML.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="41.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="10" t="s">
         <v>296</v>
       </c>
@@ -4911,13 +5332,20 @@
         <f aca="false">IF(K55="","",LEN(K55))</f>
         <v>39</v>
       </c>
-      <c r="M55" s="13" t="s">
-        <v>63</v>
+      <c r="M55" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N55" s="13"/>
-      <c r="O55" s="13"/>
-    </row>
-    <row r="56" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O55" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the page title is set in the page's own metadata (src/lib/seo.ts pageMetadata). No change needed.
+Checked live 9 Oct 2026: title is 'RFID Product Categories | Virtualsphere' (39 chars).</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="54.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="10" t="s">
         <v>302</v>
       </c>
@@ -4956,13 +5384,20 @@
         <f aca="false">IF(K56="","",LEN(K56))</f>
         <v>53</v>
       </c>
-      <c r="M56" s="13" t="s">
-        <v>63</v>
+      <c r="M56" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N56" s="13"/>
-      <c r="O56" s="13"/>
-    </row>
-    <row r="57" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O56" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the page title is set in the page's own metadata (src/lib/seo.ts pageMetadata). No change needed.
+Checked live 9 Oct 2026: title is 'About Us – RFID Manufacturer in India | Virtualsphere' (53 chars).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="54.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="10" t="s">
         <v>308</v>
       </c>
@@ -5001,11 +5436,18 @@
         <f aca="false">IF(K57="","",LEN(K57))</f>
         <v>50</v>
       </c>
-      <c r="M57" s="13" t="s">
-        <v>63</v>
+      <c r="M57" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N57" s="13"/>
-      <c r="O57" s="13"/>
+      <c r="O57" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the page title is set in the page's own metadata (src/lib/seo.ts pageMetadata). No change needed.
+Checked live 9 Oct 2026: title is 'Contact Us – RFID Quotes &amp; Support | Virtualsphere' (50 chars).</t>
+        </is>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="10" t="s">
@@ -5040,13 +5482,24 @@
       </c>
       <c r="K58" s="10"/>
       <c r="L58" s="12"/>
-      <c r="M58" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N58" s="13"/>
-      <c r="O58" s="13"/>
-    </row>
-    <row r="59" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M58" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N58" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O58" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: page heading (H1) changed from 'Get in touch' to 'Contact Virtualsphere' (src/app/(public)/contact/page.tsx, commit c912301, deployed); the small label above it now reads 'Get in touch'. The 'India RFID shop...' text is an H2 sub-heading in the page source, not an H1.
+Verified live: the page has exactly one H1: 'Contact Virtualsphere'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="54.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="10" t="s">
         <v>318</v>
       </c>
@@ -5085,13 +5538,24 @@
         <f aca="false">IF(K59="","",LEN(K59))</f>
         <v>50</v>
       </c>
-      <c r="M59" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N59" s="13"/>
-      <c r="O59" s="13"/>
-    </row>
-    <row r="60" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M59" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N59" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O59" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: SEO title (Meta Title) changed in the live catalog from 'RFID Cable Tie Tags | UHF, HF &amp; LF Asset Tracking Tags' to 'RFID Cable Tie Tags – UHF, HF &amp; LF' (brand is added by the site, so 50 chars in Google).
+Verified live: page &lt;title&gt; reads 'RFID Cable Tie Tags – UHF, HF &amp; LF | Virtualsphere'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="54.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="10" t="s">
         <v>325</v>
       </c>
@@ -5130,13 +5594,24 @@
         <f aca="false">IF(K60="","",LEN(K60))</f>
         <v>55</v>
       </c>
-      <c r="M60" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N60" s="13"/>
-      <c r="O60" s="13"/>
-    </row>
-    <row r="61" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M60" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N60" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O60" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: SEO title (Meta Title) changed in the live catalog from 'RFID Laundry Silicon Tags | Washable UHF Textile RFID Tags' to 'RFID Laundry Silicon Tags, Washable UHF' (brand is added by the site, so 55 chars in Google).
+Verified live: page &lt;title&gt; reads 'RFID Laundry Silicon Tags, Washable UHF | Virtualsphere'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="54.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="10" t="s">
         <v>330</v>
       </c>
@@ -5175,13 +5650,24 @@
         <f aca="false">IF(K61="","",LEN(K61))</f>
         <v>52</v>
       </c>
-      <c r="M61" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N61" s="13"/>
-      <c r="O61" s="13"/>
-    </row>
-    <row r="62" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M61" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N61" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O61" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: SEO title (Meta Title) changed in the live catalog from 'RFID Ferric 100 Metal Tags | UHF ABS On-Metal RFID Tags' to 'VS Ferric-100 UHF On-Metal RFID Tags' (brand is added by the site, so 52 chars in Google).
+Verified live: page &lt;title&gt; reads 'VS Ferric-100 UHF On-Metal RFID Tags | Virtualsphere'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="54.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="10" t="s">
         <v>335</v>
       </c>
@@ -5220,13 +5706,24 @@
         <f aca="false">IF(K62="","",LEN(K62))</f>
         <v>52</v>
       </c>
-      <c r="M62" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N62" s="13"/>
-      <c r="O62" s="13"/>
-    </row>
-    <row r="63" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M62" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N62" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O62" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: SEO title (Meta Title) changed in the live catalog from 'VSL-A1 RFID Fixed Reader | Android UHF RFID Reader' to 'VSL-A1 Android UHF RFID Fixed Reader' (brand is added by the site, so 52 chars in Google).
+Verified live: page &lt;title&gt; reads 'VSL-A1 Android UHF RFID Fixed Reader | Virtualsphere'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="54.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="10" t="s">
         <v>340</v>
       </c>
@@ -5265,13 +5762,24 @@
         <f aca="false">IF(K63="","",LEN(K63))</f>
         <v>50</v>
       </c>
-      <c r="M63" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N63" s="13"/>
-      <c r="O63" s="13"/>
-    </row>
-    <row r="64" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M63" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N63" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O63" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: SEO title (Meta Title) changed in the live catalog from 'VST-9662 RFID UHF Labels | Printable Higgs-3 Tags' to 'VST-9662 Printable UHF RFID Labels' (brand is added by the site, so 50 chars in Google).
+Verified live: page &lt;title&gt; reads 'VST-9662 Printable UHF RFID Labels | Virtualsphere'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="54.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="10" t="s">
         <v>345</v>
       </c>
@@ -5310,13 +5818,24 @@
         <f aca="false">IF(K64="","",LEN(K64))</f>
         <v>55</v>
       </c>
-      <c r="M64" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N64" s="13"/>
-      <c r="O64" s="13"/>
-    </row>
-    <row r="65" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M64" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N64" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O64" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: SEO title (Meta Title) changed in the live catalog from 'RFID Laundry Textile Tags | Washable UHF Fabric RFID Tags' to 'RFID Laundry Textile Tags, Washable UHF' (brand is added by the site, so 55 chars in Google).
+Verified live: page &lt;title&gt; reads 'RFID Laundry Textile Tags, Washable UHF | Virtualsphere'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="54.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="10" t="s">
         <v>350</v>
       </c>
@@ -5355,13 +5874,24 @@
         <f aca="false">IF(K65="","",LEN(K65))</f>
         <v>54</v>
       </c>
-      <c r="M65" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N65" s="13"/>
-      <c r="O65" s="13"/>
-    </row>
-    <row r="66" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M65" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N65" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O65" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: SEO title (Meta Title) changed in the live catalog from 'VST-9640 RFID UHF Inlays | Slim 98×12 mm Higgs-3 Tag' to 'VST-9640 Slim UHF RFID Inlays, Higgs-3' (brand is added by the site, so 54 chars in Google).
+Verified live: page &lt;title&gt; reads 'VST-9640 Slim UHF RFID Inlays, Higgs-3 | Virtualsphere'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="54.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="10" t="s">
         <v>355</v>
       </c>
@@ -5400,13 +5930,24 @@
         <f aca="false">IF(K66="","",LEN(K66))</f>
         <v>52</v>
       </c>
-      <c r="M66" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N66" s="13"/>
-      <c r="O66" s="13"/>
-    </row>
-    <row r="67" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M66" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N66" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O66" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: SEO title (Meta Title) changed in the live catalog from 'Dogbone RFID UHF Inlays | Impinj M730 Tag, 15 m Range' to 'Dogbone UHF RFID Inlays, Impinj M730' (brand is added by the site, so 52 chars in Google).
+Verified live: page &lt;title&gt; reads 'Dogbone UHF RFID Inlays, Impinj M730 | Virtualsphere'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="54.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="10" t="s">
         <v>360</v>
       </c>
@@ -5445,13 +5986,20 @@
         <f aca="false">IF(K67="","",LEN(K67))</f>
         <v>52</v>
       </c>
-      <c r="M67" s="13" t="s">
-        <v>63</v>
+      <c r="M67" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
       <c r="N67" s="13"/>
-      <c r="O67" s="13"/>
-    </row>
-    <row r="68" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O67" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already fixed before 9 Oct 2026 (commit 09f194b, 7 Oct): the title is set in PRODUCT_TITLES (src/app/(public)/products/[slug]/page.tsx). No change needed.
+Checked live 9 Oct 2026: title is 'UA12 12dBi Circular UHF RFID Antenna | Virtualsphere' (52 chars).</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="67.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="10" t="s">
         <v>361</v>
       </c>
@@ -5490,11 +6038,22 @@
         <f aca="false">IF(K68="","",LEN(K68))</f>
         <v>59</v>
       </c>
-      <c r="M68" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N68" s="13"/>
-      <c r="O68" s="13"/>
+      <c r="M68" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N68" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O68" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: SEO title (Meta Title) changed in the live catalog from 'RFID HRP 70 HF Pendrive reader' to 'HRP 70 13.56MHz HF RFID USB Pendrive Reader' (brand is added by the site, so 59 chars in Google).
+Verified live: page &lt;title&gt; reads 'HRP 70 13.56MHz HF RFID USB Pendrive Reader | Virtualsphere'.</t>
+        </is>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="10" t="s">
@@ -5535,13 +6094,24 @@
         <f aca="false">IF(K69="","",LEN(K69))</f>
         <v>47</v>
       </c>
-      <c r="M69" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N69" s="13"/>
-      <c r="O69" s="13"/>
-    </row>
-    <row r="70" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M69" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N69" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O69" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: SEO title (Meta Title) changed in the live catalog from 'RFID Handheld Reader | UHR 72' to 'UHR 72 UHF RFID Handheld Reader' (brand is added by the site, so 47 chars in Google).
+Verified live: page &lt;title&gt; reads 'UHR 72 UHF RFID Handheld Reader | Virtualsphere'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="67.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="10" t="s">
         <v>369</v>
       </c>
@@ -5580,13 +6150,24 @@
         <f aca="false">IF(K70="","",LEN(K70))</f>
         <v>59</v>
       </c>
-      <c r="M70" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N70" s="13"/>
-      <c r="O70" s="13"/>
-    </row>
-    <row r="71" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M70" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N70" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O70" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: SEO title (Meta Title) changed in the live catalog from 'UDM9R UHF Integrated Reader' to 'UDM9R Long Range Integrated UHF RFID Reader' (brand is added by the site, so 59 chars in Google).
+Verified live: page &lt;title&gt; reads 'UDM9R Long Range Integrated UHF RFID Reader | Virtualsphere'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="54.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="10" t="s">
         <v>373</v>
       </c>
@@ -5625,13 +6206,24 @@
         <f aca="false">IF(K71="","",LEN(K71))</f>
         <v>56</v>
       </c>
-      <c r="M71" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N71" s="13"/>
-      <c r="O71" s="13"/>
-    </row>
-    <row r="72" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M71" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N71" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O71" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: SEO title (Meta Title) changed in the live catalog from 'UDM12R UHF Integrated Reader' to 'UDM12R Impinj Integrated UHF RFID Reader' (brand is added by the site, so 56 chars in Google).
+Verified live: page &lt;title&gt; reads 'UDM12R Impinj Integrated UHF RFID Reader | Virtualsphere'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="54.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="10" t="s">
         <v>377</v>
       </c>
@@ -5670,13 +6262,24 @@
         <f aca="false">IF(K72="","",LEN(K72))</f>
         <v>58</v>
       </c>
-      <c r="M72" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N72" s="13"/>
-      <c r="O72" s="13"/>
-    </row>
-    <row r="73" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M72" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N72" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O72" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: SEO title (Meta Title) changed in the live catalog from 'Long Range RFID Reader | UDR 107' to 'UDR 107 Long Range UHF RFID Desktop Reader' (brand is added by the site, so 58 chars in Google).
+Verified live: page &lt;title&gt; reads 'UDR 107 Long Range UHF RFID Desktop Reader | Virtualsphere'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="67.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="10" t="s">
         <v>381</v>
       </c>
@@ -5709,11 +6312,22 @@
       </c>
       <c r="K73" s="10"/>
       <c r="L73" s="12"/>
-      <c r="M73" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N73" s="13"/>
-      <c r="O73" s="13"/>
+      <c r="M73" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N73" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O73" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: product name (the H1) changed in the live catalog from 'UDR 105' to 'UDR-W105 UHF RFID Desktop Reader &amp; Writer', matching the page title. The Model field was also changed from 'UDR 105' to 'UDR-W105' so the details table matches; chosen by the site owner.
+Verified live: exactly one H1: 'UDR-W105 UHF RFID Desktop Reader &amp; Writer'; page title 'UDR-W105 UHF RFID Desktop Reader &amp; Writer | Virtualsphere'.</t>
+        </is>
+      </c>
     </row>
     <row r="74" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="10" t="s">
@@ -5748,11 +6362,22 @@
       </c>
       <c r="K74" s="10"/>
       <c r="L74" s="12"/>
-      <c r="M74" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="N74" s="13"/>
-      <c r="O74" s="13"/>
+      <c r="M74" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="N74" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Claude Code</t>
+        </is>
+      </c>
+      <c r="O74" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 Oct 2026: product name (the H1) changed in the live catalog from 'RFID SILICON TAG' to 'RFID Laundry Silicon Tags', matching the page title.
+Verified live: exactly one H1: 'RFID Laundry Silicon Tags'; page title 'RFID Laundry Silicon Tags, Washable UHF | Virtualsphere'.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O74"/>
@@ -5955,11 +6580,11 @@
       </c>
       <c r="J2" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C2,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K2" s="10" t="str">
         <f aca="false">IF(J2&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5997,11 +6622,11 @@
       </c>
       <c r="J3" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C3,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K3" s="10" t="str">
         <f aca="false">IF(J3&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6039,11 +6664,11 @@
       </c>
       <c r="J4" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C4,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" s="10" t="str">
         <f aca="false">IF(J4&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6081,11 +6706,11 @@
       </c>
       <c r="J5" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C5,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K5" s="10" t="str">
         <f aca="false">IF(J5&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6123,11 +6748,11 @@
       </c>
       <c r="J6" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C6,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K6" s="10" t="str">
         <f aca="false">IF(J6&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6165,11 +6790,11 @@
       </c>
       <c r="J7" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C7,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K7" s="10" t="str">
         <f aca="false">IF(J7&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6207,11 +6832,11 @@
       </c>
       <c r="J8" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C8,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K8" s="10" t="str">
         <f aca="false">IF(J8&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6249,11 +6874,11 @@
       </c>
       <c r="J9" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C9,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" s="10" t="str">
         <f aca="false">IF(J9&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6291,11 +6916,11 @@
       </c>
       <c r="J10" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C10,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" s="10" t="str">
         <f aca="false">IF(J10&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6333,11 +6958,11 @@
       </c>
       <c r="J11" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C11,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11" s="10" t="str">
         <f aca="false">IF(J11&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6375,11 +7000,11 @@
       </c>
       <c r="J12" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C12,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K12" s="10" t="str">
         <f aca="false">IF(J12&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6417,11 +7042,11 @@
       </c>
       <c r="J13" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C13,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K13" s="10" t="str">
         <f aca="false">IF(J13&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6459,11 +7084,11 @@
       </c>
       <c r="J14" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C14,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K14" s="10" t="str">
         <f aca="false">IF(J14&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6501,11 +7126,11 @@
       </c>
       <c r="J15" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C15,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15" s="10" t="str">
         <f aca="false">IF(J15&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6543,11 +7168,11 @@
       </c>
       <c r="J16" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C16,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K16" s="10" t="str">
         <f aca="false">IF(J16&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6585,11 +7210,11 @@
       </c>
       <c r="J17" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C17,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K17" s="10" t="str">
         <f aca="false">IF(J17&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6627,11 +7252,11 @@
       </c>
       <c r="J18" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C18,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18" s="10" t="str">
         <f aca="false">IF(J18&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6669,11 +7294,11 @@
       </c>
       <c r="J19" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C19,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K19" s="10" t="str">
         <f aca="false">IF(J19&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6711,11 +7336,11 @@
       </c>
       <c r="J20" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C20,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K20" s="10" t="str">
         <f aca="false">IF(J20&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6753,11 +7378,11 @@
       </c>
       <c r="J21" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C21,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K21" s="10" t="str">
         <f aca="false">IF(J21&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6795,11 +7420,11 @@
       </c>
       <c r="J22" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C22,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K22" s="10" t="str">
         <f aca="false">IF(J22&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6837,11 +7462,11 @@
       </c>
       <c r="J23" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C23,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K23" s="10" t="str">
         <f aca="false">IF(J23&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6879,11 +7504,11 @@
       </c>
       <c r="J24" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C24,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K24" s="10" t="str">
         <f aca="false">IF(J24&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6921,11 +7546,11 @@
       </c>
       <c r="J25" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C25,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K25" s="10" t="str">
         <f aca="false">IF(J25&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6963,11 +7588,11 @@
       </c>
       <c r="J26" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C26,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K26" s="10" t="str">
         <f aca="false">IF(J26&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7005,11 +7630,11 @@
       </c>
       <c r="J27" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C27,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27" s="10" t="str">
         <f aca="false">IF(J27&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7047,11 +7672,11 @@
       </c>
       <c r="J28" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C28,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K28" s="10" t="str">
         <f aca="false">IF(J28&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7089,11 +7714,11 @@
       </c>
       <c r="J29" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C29,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K29" s="10" t="str">
         <f aca="false">IF(J29&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7131,11 +7756,11 @@
       </c>
       <c r="J30" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C30,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K30" s="10" t="str">
         <f aca="false">IF(J30&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7173,11 +7798,11 @@
       </c>
       <c r="J31" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C31,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K31" s="10" t="str">
         <f aca="false">IF(J31&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7215,11 +7840,11 @@
       </c>
       <c r="J32" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C32,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K32" s="10" t="str">
         <f aca="false">IF(J32&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7257,11 +7882,11 @@
       </c>
       <c r="J33" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C33,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K33" s="10" t="str">
         <f aca="false">IF(J33&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7299,11 +7924,11 @@
       </c>
       <c r="J34" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C34,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K34" s="10" t="str">
         <f aca="false">IF(J34&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7341,11 +7966,11 @@
       </c>
       <c r="J35" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C35,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K35" s="10" t="str">
         <f aca="false">IF(J35&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7383,11 +8008,11 @@
       </c>
       <c r="J36" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C36,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K36" s="10" t="str">
         <f aca="false">IF(J36&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7425,11 +8050,11 @@
       </c>
       <c r="J37" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C37,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K37" s="10" t="str">
         <f aca="false">IF(J37&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7467,11 +8092,11 @@
       </c>
       <c r="J38" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C38,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K38" s="10" t="str">
         <f aca="false">IF(J38&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7509,11 +8134,11 @@
       </c>
       <c r="J39" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C39,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K39" s="10" t="str">
         <f aca="false">IF(J39&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7551,11 +8176,11 @@
       </c>
       <c r="J40" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C40,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K40" s="10" t="str">
         <f aca="false">IF(J40&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7593,11 +8218,11 @@
       </c>
       <c r="J41" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C41,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K41" s="10" t="str">
         <f aca="false">IF(J41&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7635,11 +8260,11 @@
       </c>
       <c r="J42" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C42,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K42" s="10" t="str">
         <f aca="false">IF(J42&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7677,11 +8302,11 @@
       </c>
       <c r="J43" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C43,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K43" s="10" t="str">
         <f aca="false">IF(J43&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7719,11 +8344,11 @@
       </c>
       <c r="J44" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C44,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K44" s="10" t="str">
         <f aca="false">IF(J44&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7761,11 +8386,11 @@
       </c>
       <c r="J45" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C45,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K45" s="10" t="str">
         <f aca="false">IF(J45&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7803,11 +8428,11 @@
       </c>
       <c r="J46" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C46,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K46" s="10" t="str">
         <f aca="false">IF(J46&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7845,11 +8470,11 @@
       </c>
       <c r="J47" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C47,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K47" s="10" t="str">
         <f aca="false">IF(J47&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7887,11 +8512,11 @@
       </c>
       <c r="J48" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C48,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K48" s="10" t="str">
         <f aca="false">IF(J48&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7971,11 +8596,11 @@
       </c>
       <c r="J50" s="10" t="n">
         <f aca="false">COUNTIFS(Issues!$E$2:$E$74,C50,Issues!$M$2:$M$74,"&lt;&gt;Fixed",Issues!$M$2:$M$74,"&lt;&gt;Verified")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K50" s="10" t="str">
         <f aca="false">IF(J50&gt;0,"Needs fix","OK")</f>
-        <v>Needs fix</v>
+        <v>OK</v>
       </c>
     </row>
   </sheetData>

</xml_diff>